<commit_message>
Update Grove Sensor Inventory.xlsx
</commit_message>
<xml_diff>
--- a/GoPiGo3 Documentation/Sensors/Grove Sensor Inventory.xlsx
+++ b/GoPiGo3 Documentation/Sensors/Grove Sensor Inventory.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB159DB-3918-4F3E-84BB-6C717B487CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AAC7A3-A497-482E-B3CF-CFE4E2A35C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30120" yWindow="3740" windowWidth="28800" windowHeight="15460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30120" yWindow="3740" windowWidth="28800" windowHeight="15460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grove Sensor Inventory" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="81">
   <si>
     <t>Future Purchases</t>
   </si>
@@ -236,6 +236,42 @@
   </si>
   <si>
     <t>Raspberry Pi 3</t>
+  </si>
+  <si>
+    <t>Light and Color Sensor</t>
+  </si>
+  <si>
+    <t>Inertial Measurement Unit</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Camera V2</t>
+  </si>
+  <si>
+    <t>Grove - Buzzer</t>
+  </si>
+  <si>
+    <t>Hamburger Mini Speaker</t>
+  </si>
+  <si>
+    <t>IR Remote Control</t>
+  </si>
+  <si>
+    <t>Grove - Infrared Receiver</t>
+  </si>
+  <si>
+    <t>Grove - Air Quality Sensor</t>
+  </si>
+  <si>
+    <t>Grove - Dust Sensor</t>
+  </si>
+  <si>
+    <t>Pixycam's</t>
+  </si>
+  <si>
+    <t>MakerFocus IR Camera's and Mount</t>
+  </si>
+  <si>
+    <t>GoPiGo Servos</t>
   </si>
 </sst>
 </file>
@@ -588,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.453125" customWidth="1"/>
@@ -781,22 +817,20 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>4</v>
+      </c>
       <c r="B21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -887,72 +921,189 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B34" s="1" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="4"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="4"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="4"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>2</v>
+      </c>
+      <c r="B43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B47" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B35" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B48" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B36" t="s">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B49" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B37" t="s">
+      <c r="C49" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B38" t="s">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B51" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C51" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B39" t="s">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B52" t="s">
         <v>46</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B40" t="s">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B53" t="s">
         <v>48</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B41" t="s">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B54" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B42" t="s">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
         <v>52</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -968,7 +1119,7 @@
     <hyperlink ref="C10" r:id="rId8" xr:uid="{891D535F-ADF2-4D13-B620-A73668B2015A}"/>
     <hyperlink ref="C11" r:id="rId9" xr:uid="{AC7142FE-E266-4CD3-97DB-1310842B0B61}"/>
     <hyperlink ref="C20" r:id="rId10" xr:uid="{A073B9A2-DBB1-4AF0-9A2F-62F771977C1F}"/>
-    <hyperlink ref="C21" r:id="rId11" xr:uid="{2D5B5A2C-D5B6-4588-AEE3-8ECFA75C1201}"/>
+    <hyperlink ref="C22" r:id="rId11" xr:uid="{2D5B5A2C-D5B6-4588-AEE3-8ECFA75C1201}"/>
     <hyperlink ref="C15" r:id="rId12" xr:uid="{FCBD3AAD-59EE-4F08-9175-80EEFCACB33F}"/>
     <hyperlink ref="C16" r:id="rId13" xr:uid="{9C40FB68-FD8A-4B09-8F17-6844C7A9D571}"/>
     <hyperlink ref="C17" r:id="rId14" xr:uid="{12E0AEC3-3D8E-4808-BFAB-59E5419EC290}"/>
@@ -977,24 +1128,23 @@
     <hyperlink ref="C13" r:id="rId17" xr:uid="{B1890AE7-704D-4F7F-A435-82067556A9C1}"/>
     <hyperlink ref="C14" r:id="rId18" xr:uid="{8FB09DF9-26F4-459D-8571-66D1144A7692}"/>
     <hyperlink ref="C19" r:id="rId19" xr:uid="{8DFCF142-5A15-4491-8B41-8E5DCA79F9D6}"/>
-    <hyperlink ref="C36" r:id="rId20" xr:uid="{1F4B886A-07F1-402D-BCD6-9D21FBC22F79}"/>
-    <hyperlink ref="C35" r:id="rId21" xr:uid="{47E231DF-3D24-46C5-8A70-4694A0A42CD4}"/>
-    <hyperlink ref="C37" r:id="rId22" xr:uid="{80C35267-0878-489A-BFF1-A40671AB2374}"/>
-    <hyperlink ref="C39" r:id="rId23" xr:uid="{F081FC22-55F9-4C01-B2BE-E0E26F57C0D5}"/>
-    <hyperlink ref="C40" r:id="rId24" xr:uid="{65EB04FA-9093-4791-8530-37E443B5B138}"/>
-    <hyperlink ref="C41" r:id="rId25" display="https://www.amazon.com/dp/B007OYAVLI/ref=sspa_dk_detail_3?psc=1&amp;pd_rd_i=B007OYAVLI&amp;pd_rd_w=SWp2j&amp;content-id=amzn1.sym.248b5e31-60e8-4934-96cf-b3789198461a&amp;pf_rd_p=248b5e31-60e8-4934-96cf-b3789198461a&amp;pf_rd_r=G9XKB7F7ZW32SHGXCAHB&amp;pd_rd_wg=vmZm9&amp;pd_rd_r=e57e8e71-7e40-4fa7-b01b-b011b28916fd&amp;s=electronics&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9kZXRhaWxfdGhlbWF0aWM" xr:uid="{31B86A5B-33D7-4897-8770-3263ADFFD1EF}"/>
-    <hyperlink ref="C42" r:id="rId26" display="https://www.amazon.com/youyeetoo-Triangular-Raspberry-Avoidance-Navigation/dp/B0B77F4S9H/ref=sr_1_1?dib=eyJ2IjoiMSJ9.rFlCxHNbPw8BWyOn2IUEhSGJU0MFt8TYGUMRznzGnjk.BbFwUPRtHEpoJuVKVxLFCT67NG3_jzJ_XwHLdP3pyXM&amp;dib_tag=se&amp;hvadid=410084536784&amp;hvdev=c&amp;hvlocphy=9025095&amp;hvnetw=g&amp;hvqmt=e&amp;hvrand=9041788616229778693&amp;hvtargid=kwd-649296963536&amp;hydadcr=10893_11286874&amp;keywords=ydlidar+x4&amp;qid=1715704804&amp;sr=8-1" xr:uid="{E2E1859A-D213-4DA3-800E-68D72D46FF94}"/>
-    <hyperlink ref="C38" r:id="rId27" xr:uid="{9B95F973-70EF-42BD-B3BB-A6858198C45B}"/>
-    <hyperlink ref="C22" r:id="rId28" xr:uid="{31D839AF-3DAE-4801-B0A9-4AED74451AE8}"/>
-    <hyperlink ref="C26" r:id="rId29" xr:uid="{0380BA65-C202-4026-A5CE-EEE2E88D5190}"/>
-    <hyperlink ref="C27" r:id="rId30" xr:uid="{0C62F906-35A5-4C8D-A9BD-54505798D95B}"/>
-    <hyperlink ref="C29" r:id="rId31" display="https://www.seeedstudio.com/Grove-Base-Hat-for-Raspberry-Pi.html" xr:uid="{1597AFFD-00AC-4D89-8E4F-C63C2CE23695}"/>
-    <hyperlink ref="C24" r:id="rId32" xr:uid="{81088FD7-C84E-4216-8DF6-213B37D1BAB8}"/>
-    <hyperlink ref="C23" r:id="rId33" xr:uid="{6CCDEB82-4E33-4806-8E29-085B40F4E59C}"/>
-    <hyperlink ref="C25" r:id="rId34" xr:uid="{91276966-46A8-4892-B2CD-3127DA180536}"/>
+    <hyperlink ref="C49" r:id="rId20" xr:uid="{1F4B886A-07F1-402D-BCD6-9D21FBC22F79}"/>
+    <hyperlink ref="C48" r:id="rId21" xr:uid="{47E231DF-3D24-46C5-8A70-4694A0A42CD4}"/>
+    <hyperlink ref="C50" r:id="rId22" xr:uid="{80C35267-0878-489A-BFF1-A40671AB2374}"/>
+    <hyperlink ref="C52" r:id="rId23" xr:uid="{F081FC22-55F9-4C01-B2BE-E0E26F57C0D5}"/>
+    <hyperlink ref="C53" r:id="rId24" xr:uid="{65EB04FA-9093-4791-8530-37E443B5B138}"/>
+    <hyperlink ref="C54" r:id="rId25" display="https://www.amazon.com/dp/B007OYAVLI/ref=sspa_dk_detail_3?psc=1&amp;pd_rd_i=B007OYAVLI&amp;pd_rd_w=SWp2j&amp;content-id=amzn1.sym.248b5e31-60e8-4934-96cf-b3789198461a&amp;pf_rd_p=248b5e31-60e8-4934-96cf-b3789198461a&amp;pf_rd_r=G9XKB7F7ZW32SHGXCAHB&amp;pd_rd_wg=vmZm9&amp;pd_rd_r=e57e8e71-7e40-4fa7-b01b-b011b28916fd&amp;s=electronics&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9kZXRhaWxfdGhlbWF0aWM" xr:uid="{31B86A5B-33D7-4897-8770-3263ADFFD1EF}"/>
+    <hyperlink ref="C55" r:id="rId26" display="https://www.amazon.com/youyeetoo-Triangular-Raspberry-Avoidance-Navigation/dp/B0B77F4S9H/ref=sr_1_1?dib=eyJ2IjoiMSJ9.rFlCxHNbPw8BWyOn2IUEhSGJU0MFt8TYGUMRznzGnjk.BbFwUPRtHEpoJuVKVxLFCT67NG3_jzJ_XwHLdP3pyXM&amp;dib_tag=se&amp;hvadid=410084536784&amp;hvdev=c&amp;hvlocphy=9025095&amp;hvnetw=g&amp;hvqmt=e&amp;hvrand=9041788616229778693&amp;hvtargid=kwd-649296963536&amp;hydadcr=10893_11286874&amp;keywords=ydlidar+x4&amp;qid=1715704804&amp;sr=8-1" xr:uid="{E2E1859A-D213-4DA3-800E-68D72D46FF94}"/>
+    <hyperlink ref="C51" r:id="rId27" xr:uid="{9B95F973-70EF-42BD-B3BB-A6858198C45B}"/>
+    <hyperlink ref="C26" r:id="rId28" xr:uid="{0380BA65-C202-4026-A5CE-EEE2E88D5190}"/>
+    <hyperlink ref="C27" r:id="rId29" xr:uid="{0C62F906-35A5-4C8D-A9BD-54505798D95B}"/>
+    <hyperlink ref="C29" r:id="rId30" display="https://www.seeedstudio.com/Grove-Base-Hat-for-Raspberry-Pi.html" xr:uid="{1597AFFD-00AC-4D89-8E4F-C63C2CE23695}"/>
+    <hyperlink ref="C24" r:id="rId31" xr:uid="{81088FD7-C84E-4216-8DF6-213B37D1BAB8}"/>
+    <hyperlink ref="C23" r:id="rId32" xr:uid="{6CCDEB82-4E33-4806-8E29-085B40F4E59C}"/>
+    <hyperlink ref="C25" r:id="rId33" xr:uid="{91276966-46A8-4892-B2CD-3127DA180536}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId35"/>
+  <pageSetup orientation="portrait" r:id="rId34"/>
 </worksheet>
 </file>
 

</xml_diff>